<commit_message>
Tax List,Promocode List,Cancellation Policy List , Aminities List, Other Payment Entry and List Master Added
</commit_message>
<xml_diff>
--- a/src/HotelRestaurant.Infrastructure/SQL/MasterData.xlsx
+++ b/src/HotelRestaurant.Infrastructure/SQL/MasterData.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet3" sheetId="3" r:id="rId1"/>
     <sheet name="Room" sheetId="1" r:id="rId2"/>
     <sheet name="RoomTYpes" sheetId="2" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
@@ -1920,4 +1921,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>